<commit_message>
scripts para anadir data de grupos 1 y 6
</commit_message>
<xml_diff>
--- a/consultas_graficas.xlsx
+++ b/consultas_graficas.xlsx
@@ -30,7 +30,7 @@
     <font>
       <b val="1"/>
       <color rgb="002F5496"/>
-      <sz val="14"/>
+      <sz val="13"/>
     </font>
     <font>
       <b val="1"/>
@@ -78,9 +78,7 @@
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -168,373 +166,31 @@
 </styleSheet>
 </file>
 
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Citas por Especialidad Médica</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="bar"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Citas por Especialidad'!B3</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="2F5496"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Citas por Especialidad'!$A$4:$A$18</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Citas por Especialidad'!$B$4:$B$18</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Cantidad de Citas</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Especialidad</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Citas Médicas por Mes (Estacionalidad)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Citas por Mes'!B3</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25000">
-              <a:solidFill>
-                <a:srgbClr val="2F5496"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Citas por Mes'!$A$4:$A$28</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Citas por Mes'!$B$4:$B$28</f>
-            </numRef>
-          </val>
-        </ser>
-        <axId val="10"/>
-        <axId val="100"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Mes</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Cantidad de Citas</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Diagnósticos por Tipo</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="bar"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Diagnósticos por Tipo'!B3</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="C55A11"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Diagnósticos por Tipo'!$A$4:$A$26</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Diagnósticos por Tipo'!$B$4:$B$26</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Cantidad</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Tipo de Diagnóstico</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>3</col>
       <colOff>0</colOff>
-      <row>2</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7920000" cy="5040000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
+    <ext cx="14287500" cy="8572500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
     <clientData/>
   </oneCellAnchor>
 </wsDr>
@@ -546,22 +202,25 @@
     <from>
       <col>3</col>
       <colOff>0</colOff>
-      <row>2</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10080000" cy="5040000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
+    <ext cx="17145000" cy="7143750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
     <clientData/>
   </oneCellAnchor>
 </wsDr>
@@ -573,22 +232,25 @@
     <from>
       <col>3</col>
       <colOff>0</colOff>
-      <row>2</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8640000" cy="6480000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
+    <ext cx="14287500" cy="11430000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
     <clientData/>
   </oneCellAnchor>
 </wsDr>
@@ -1060,9 +722,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -1351,9 +1010,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -1622,9 +1278,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>